<commit_message>
fix(perf): correct FP4 peak and MFU metrics
</commit_message>
<xml_diff>
--- a/eval/perf_data/operator_performance_full_list_20261010_styled_headers_matmul_reuseA.xlsx
+++ b/eval/perf_data/operator_performance_full_list_20261010_styled_headers_matmul_reuseA.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markdown完整列表" sheetId="1" r:id="R8f665c5daf534bd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FA_FP8_BF16_Tk择优" sheetId="3" r:id="R62cc71e0627148b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matmul原始数据" sheetId="4" r:id="R67538ccb302a4091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markdown完整列表" sheetId="1" r:id="R01ac29ef71104e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FA_FP8_BF16_Tk择优" sheetId="3" r:id="R39ee05a830af450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matmul原始数据" sheetId="4" r:id="R9ea6637c43e04d98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3923,7 +3923,7 @@
         <x:v>峰值 FMA/cycle</x:v>
       </x:c>
       <x:c r="B6" s="274" t="str">
-        <x:v>BF16=4096; FP8=8192; MXFP4=16384 FMA/cycle（与 gfsim Cube PMU 口径一致）</x:v>
+        <x:v>BF16=4096; FP8=8192; MXFP4/HIF4=32768 FMA/cycle（峰值比 1:2:8）</x:v>
       </x:c>
       <x:c r="C6" s="363"/>
       <x:c r="D6" s="366" t="str">
@@ -4111,15 +4111,15 @@
         <x:v>224.0425</x:v>
       </x:c>
       <x:c r="K10" s="868" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L10" s="868" t="n">
         <x:f>IF(I10="","",2*128*65536*D10/K10)</x:f>
-        <x:v>262144</x:v>
+        <x:v>131072</x:v>
       </x:c>
       <x:c r="M10" s="867" t="n">
         <x:f>IF(I10="","",L10/I10)</x:f>
-        <x:v>0.7312898222435475</x:v>
+        <x:v>0.3656449111217738</x:v>
       </x:c>
       <x:c r="N10" s="870" t="n">
         <x:f>IF(J10="","",J10/G10)</x:f>
@@ -4164,7 +4164,7 @@
       <x:c r="I11" s="873"/>
       <x:c r="J11" s="874"/>
       <x:c r="K11" s="873" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L11" s="873"/>
       <x:c r="M11" s="872"/>
@@ -4213,15 +4213,15 @@
         <x:v>136.594375</x:v>
       </x:c>
       <x:c r="K12" s="873" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L12" s="873" t="n">
         <x:f>IF(I12="","",2*128*65536*D12/K12)</x:f>
-        <x:v>131072</x:v>
+        <x:v>65536</x:v>
       </x:c>
       <x:c r="M12" s="872" t="n">
         <x:f>IF(I12="","",L12/I12)</x:f>
-        <x:v>0.5997318703643543</x:v>
+        <x:v>0.29986593518217713</x:v>
       </x:c>
       <x:c r="N12" s="875" t="n">
         <x:f>IF(J12="","",J12/G12)</x:f>
@@ -4271,15 +4271,15 @@
         <x:v>77.7175</x:v>
       </x:c>
       <x:c r="K13" s="873" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L13" s="873" t="n">
         <x:f>IF(I13="","",2*128*65536*D13/K13)</x:f>
-        <x:v>65536</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="M13" s="872" t="n">
         <x:f>IF(I13="","",L13/I13)</x:f>
-        <x:v>0.5270370251230417</x:v>
+        <x:v>0.26351851256152087</x:v>
       </x:c>
       <x:c r="N13" s="875" t="n">
         <x:f>IF(J13="","",J13/G13)</x:f>
@@ -5281,15 +5281,15 @@
       </x:c>
       <x:c r="K32" s="898" t="n">
         <x:f>'Matmul原始数据'!Q54</x:f>
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L32" s="898" t="n">
         <x:f>'Matmul原始数据'!R54</x:f>
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="M32" s="906" t="n">
         <x:f>'Matmul原始数据'!S54</x:f>
-        <x:v>0.0414900185223297</x:v>
+        <x:v>0.02074500926116485</x:v>
       </x:c>
       <x:c r="N32" s="900"/>
       <x:c r="O32" s="930" t="str">
@@ -5339,15 +5339,15 @@
       </x:c>
       <x:c r="K33" s="910" t="n">
         <x:f>'Matmul原始数据'!Q58</x:f>
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="L33" s="910" t="n">
         <x:f>'Matmul原始数据'!R58</x:f>
-        <x:v>81920</x:v>
+        <x:v>40960</x:v>
       </x:c>
       <x:c r="M33" s="906" t="n">
         <x:f>'Matmul原始数据'!S58</x:f>
-        <x:v>0.2463833498751842</x:v>
+        <x:v>0.1231916749375921</x:v>
       </x:c>
       <x:c r="N33" s="912"/>
       <x:c r="O33" s="931" t="str">
@@ -11600,10 +11600,10 @@
       <x:c r="O51" s="985"/>
       <x:c r="P51" s="1010"/>
       <x:c r="Q51" s="985" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R51" s="985" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S51" s="1011"/>
       <x:c r="T51" s="1009"/>
@@ -11675,10 +11675,10 @@
       <x:c r="O52" s="985"/>
       <x:c r="P52" s="1010"/>
       <x:c r="Q52" s="985" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R52" s="985" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S52" s="1011"/>
       <x:c r="T52" s="1009"/>
@@ -11750,10 +11750,10 @@
       <x:c r="O53" s="985"/>
       <x:c r="P53" s="1010"/>
       <x:c r="Q53" s="985" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R53" s="985" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S53" s="1011"/>
       <x:c r="T53" s="1009"/>
@@ -11829,22 +11829,22 @@
         <x:v>30.36875</x:v>
       </x:c>
       <x:c r="Q54" s="998" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R54" s="998" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S54" s="1000" t="n">
-        <x:v>0.0414900185223297</x:v>
+        <x:v>0.02074500926116485</x:v>
       </x:c>
       <x:c r="T54" s="1009" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="U54" s="1009" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="V54" s="1011" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.125</x:v>
       </x:c>
       <x:c r="W54" s="701" t="str">
         <x:v>PASS</x:v>
@@ -11912,10 +11912,10 @@
       <x:c r="O55" s="985"/>
       <x:c r="P55" s="1010"/>
       <x:c r="Q55" s="985" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R55" s="985" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S55" s="1011"/>
       <x:c r="T55" s="1009"/>
@@ -11987,10 +11987,10 @@
       <x:c r="O56" s="985"/>
       <x:c r="P56" s="1010"/>
       <x:c r="Q56" s="985" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R56" s="985" t="n">
-        <x:v>2016</x:v>
+        <x:v>1008</x:v>
       </x:c>
       <x:c r="S56" s="1011"/>
       <x:c r="T56" s="1009"/>
@@ -12066,22 +12066,22 @@
         <x:v>333.711875</x:v>
       </x:c>
       <x:c r="Q57" s="986" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R57" s="986" t="n">
-        <x:v>81920</x:v>
+        <x:v>40960</x:v>
       </x:c>
       <x:c r="S57" s="1015" t="n">
-        <x:v>0.15342576586463996</x:v>
+        <x:v>0.07671288293231998</x:v>
       </x:c>
       <x:c r="T57" s="1013" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="U57" s="1013" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="V57" s="1015" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.125</x:v>
       </x:c>
       <x:c r="W57" s="709" t="str">
         <x:v>PASS</x:v>
@@ -12153,22 +12153,22 @@
         <x:v>207.80625</x:v>
       </x:c>
       <x:c r="Q58" s="998" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R58" s="998" t="n">
-        <x:v>81920</x:v>
+        <x:v>40960</x:v>
       </x:c>
       <x:c r="S58" s="1000" t="n">
-        <x:v>0.2463833498751842</x:v>
+        <x:v>0.1231916749375921</x:v>
       </x:c>
       <x:c r="T58" s="1013" t="n">
-        <x:v>384</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="U58" s="1013" t="n">
-        <x:v>256</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="V58" s="1015" t="n">
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="W58" s="709" t="str">
         <x:v>PASS</x:v>
@@ -12240,22 +12240,22 @@
         <x:v>252.288125</x:v>
       </x:c>
       <x:c r="Q59" s="986" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R59" s="986" t="n">
-        <x:v>81920</x:v>
+        <x:v>40960</x:v>
       </x:c>
       <x:c r="S59" s="1015" t="n">
-        <x:v>0.2029425681450524</x:v>
+        <x:v>0.1014712840725262</x:v>
       </x:c>
       <x:c r="T59" s="1013" t="n">
-        <x:v>384</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="U59" s="1013" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="V59" s="1015" t="n">
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="W59" s="709" t="str">
         <x:v>PASS</x:v>
@@ -12327,22 +12327,22 @@
         <x:v>236.984375</x:v>
       </x:c>
       <x:c r="Q60" s="987" t="n">
-        <x:v>16384</x:v>
+        <x:v>32768</x:v>
       </x:c>
       <x:c r="R60" s="987" t="n">
-        <x:v>81920</x:v>
+        <x:v>40960</x:v>
       </x:c>
       <x:c r="S60" s="1019" t="n">
-        <x:v>0.21604799894507812</x:v>
+        <x:v>0.10802399947253906</x:v>
       </x:c>
       <x:c r="T60" s="1017" t="n">
-        <x:v>288</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="U60" s="1017" t="n">
-        <x:v>256</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="V60" s="1019" t="n">
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.2222222222222222</x:v>
       </x:c>
       <x:c r="W60" s="727" t="str">
         <x:v>PASS</x:v>

</xml_diff>